<commit_message>
Added config.json, backup folder
</commit_message>
<xml_diff>
--- a/doubts.xlsx
+++ b/doubts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,10 +434,30 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>teacher</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>explain</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>desc</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>reply</t>
         </is>

</xml_diff>